<commit_message>
chore: include selected local merge changes
</commit_message>
<xml_diff>
--- a/fixtures/b3/complex-submission.xlsx
+++ b/fixtures/b3/complex-submission.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catatan internal" sheetId="2" state="hidden" r:id="rId2"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:workbookPr/>
+  <ns0:workbookProtection/>
+  <ns0:bookViews>
+    <ns0:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="Ringkasan" sheetId="1" state="visible" r:id="rId1"/>
+    <ns0:sheet name="Catatan internal" sheetId="2" state="hidden" r:id="rId2"/>
+    <ns0:sheet name="Rekap Nilai Semester Akademik" sheetId="3" state="visible" r:id="rId5"/>
+  </ns0:sheets>
+  <ns0:definedNames/>
+  <ns0:calcPr calcId="124519" fullCalcOnLoad="1"/>
+</ns0:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -664,4 +665,18 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Data untuk tab dengan nama panjang</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>